<commit_message>
Added second scenario beacon harbor
</commit_message>
<xml_diff>
--- a/data/Beacon_Harbor_Winds of Fortune Template.xlsx
+++ b/data/Beacon_Harbor_Winds of Fortune Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Probability Management\Portfolio Build\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED2FD44-1633-4999-8AF8-926DC0E32420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F5A095A-CC77-4201-B7A3-EBE7102BBD71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{62E0E9A3-437D-464E-8FB6-CFA38D87EB32}"/>
   </bookViews>
@@ -583,13 +583,13 @@
         <v>9</v>
       </c>
       <c r="C5" s="5">
-        <v>0.06</v>
+        <v>0.6</v>
       </c>
       <c r="D5" s="5">
-        <v>5.0000000000000001E-3</v>
+        <v>0.5</v>
       </c>
       <c r="E5" s="5">
-        <v>2.0000000000000004E-2</v>
+        <v>0.2</v>
       </c>
       <c r="F5" s="5">
         <v>0</v>
@@ -598,7 +598,7 @@
         <v>0.3</v>
       </c>
       <c r="H5" s="5">
-        <v>2.0000000000000004E-2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -606,13 +606,13 @@
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <v>6.9999999999999993E-2</v>
+        <v>0.7</v>
       </c>
       <c r="D6" s="5">
-        <v>6.0000000000000001E-3</v>
+        <v>0.6</v>
       </c>
       <c r="E6" s="5">
-        <v>2.0000000000000004E-2</v>
+        <v>0.2</v>
       </c>
       <c r="F6" s="5">
         <v>0</v>
@@ -621,7 +621,7 @@
         <v>0.1</v>
       </c>
       <c r="H6" s="5">
-        <v>2.0000000000000004E-2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -629,13 +629,13 @@
         <v>11</v>
       </c>
       <c r="C7" s="5">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="D7" s="5">
-        <v>1.2E-2</v>
+        <v>1.2</v>
       </c>
       <c r="E7" s="5">
-        <v>0.03</v>
+        <v>0.3</v>
       </c>
       <c r="F7" s="5">
         <v>0</v>
@@ -644,7 +644,7 @@
         <v>0.4</v>
       </c>
       <c r="H7" s="5">
-        <v>0.03</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -652,13 +652,13 @@
         <v>12</v>
       </c>
       <c r="C8" s="5">
-        <v>0.11000000000000001</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="D8" s="5">
-        <v>1.3000000000000001E-2</v>
+        <v>1.3</v>
       </c>
       <c r="E8" s="5">
-        <v>2.0000000000000004E-2</v>
+        <v>0.2</v>
       </c>
       <c r="F8" s="5">
         <v>0</v>
@@ -667,7 +667,7 @@
         <v>0.1</v>
       </c>
       <c r="H8" s="5">
-        <v>0.03</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -675,13 +675,13 @@
         <v>13</v>
       </c>
       <c r="C9" s="5">
-        <v>0.05</v>
+        <v>0.5</v>
       </c>
       <c r="D9" s="5">
-        <v>4.0000000000000001E-3</v>
+        <v>0.4</v>
       </c>
       <c r="E9" s="5">
-        <v>8.0000000000000016E-2</v>
+        <v>0.8</v>
       </c>
       <c r="F9" s="5">
         <v>0</v>
@@ -690,7 +690,7 @@
         <v>0.2</v>
       </c>
       <c r="H9" s="5">
-        <v>1.0000000000000002E-2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -698,13 +698,13 @@
         <v>14</v>
       </c>
       <c r="C10" s="5">
-        <v>0.06</v>
+        <v>0.6</v>
       </c>
       <c r="D10" s="5">
-        <v>5.0000000000000001E-3</v>
+        <v>0.5</v>
       </c>
       <c r="E10" s="5">
-        <v>4.0000000000000008E-2</v>
+        <v>0.4</v>
       </c>
       <c r="F10" s="5">
         <v>0</v>
@@ -713,7 +713,7 @@
         <v>0.7</v>
       </c>
       <c r="H10" s="5">
-        <v>2.0000000000000004E-2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -721,13 +721,13 @@
         <v>15</v>
       </c>
       <c r="C11" s="5">
-        <v>0.12</v>
+        <v>1.2</v>
       </c>
       <c r="D11" s="5">
-        <v>1.4999999999999999E-2</v>
+        <v>1.5</v>
       </c>
       <c r="E11" s="5">
-        <v>0.05</v>
+        <v>0.5</v>
       </c>
       <c r="F11" s="5">
         <v>0.2</v>
@@ -736,7 +736,7 @@
         <v>0.2</v>
       </c>
       <c r="H11" s="5">
-        <v>0.06</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -744,13 +744,13 @@
         <v>16</v>
       </c>
       <c r="C12" s="5">
-        <v>0.15000000000000002</v>
+        <v>1.5</v>
       </c>
       <c r="D12" s="5">
-        <v>1.8000000000000002E-2</v>
+        <v>1.8</v>
       </c>
       <c r="E12" s="5">
-        <v>0.06</v>
+        <v>0.6</v>
       </c>
       <c r="F12" s="5">
         <v>0.2</v>
@@ -759,7 +759,7 @@
         <v>0.2</v>
       </c>
       <c r="H12" s="5">
-        <v>8.0000000000000016E-2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -767,13 +767,13 @@
         <v>17</v>
       </c>
       <c r="C13" s="5">
-        <v>4.0000000000000008E-2</v>
+        <v>0.4</v>
       </c>
       <c r="D13" s="5">
-        <v>3.0000000000000001E-3</v>
+        <v>0.3</v>
       </c>
       <c r="E13" s="5">
-        <v>0.11000000000000001</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="F13" s="5">
         <v>1.3</v>
@@ -782,7 +782,7 @@
         <v>0.2</v>
       </c>
       <c r="H13" s="5">
-        <v>0.03</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -790,13 +790,13 @@
         <v>18</v>
       </c>
       <c r="C14" s="5">
-        <v>8.0000000000000016E-2</v>
+        <v>0.8</v>
       </c>
       <c r="D14" s="5">
-        <v>6.9999999999999993E-3</v>
+        <v>0.7</v>
       </c>
       <c r="E14" s="5">
-        <v>2.0000000000000004E-2</v>
+        <v>0.2</v>
       </c>
       <c r="F14" s="5">
         <v>0</v>
@@ -805,7 +805,7 @@
         <v>0.1</v>
       </c>
       <c r="H14" s="5">
-        <v>4.0000000000000008E-2</v>
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updating winds templates for scenarios
</commit_message>
<xml_diff>
--- a/data/Beacon_Harbor_Winds of Fortune Template.xlsx
+++ b/data/Beacon_Harbor_Winds of Fortune Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Probability Management\Portfolio Build\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F5A095A-CC77-4201-B7A3-EBE7102BBD71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED2FD44-1633-4999-8AF8-926DC0E32420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{62E0E9A3-437D-464E-8FB6-CFA38D87EB32}"/>
   </bookViews>
@@ -583,13 +583,13 @@
         <v>9</v>
       </c>
       <c r="C5" s="5">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
       <c r="D5" s="5">
-        <v>0.5</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="E5" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
       <c r="F5" s="5">
         <v>0</v>
@@ -598,7 +598,7 @@
         <v>0.3</v>
       </c>
       <c r="H5" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -606,13 +606,13 @@
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <v>0.7</v>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="D6" s="5">
-        <v>0.6</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="E6" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
       <c r="F6" s="5">
         <v>0</v>
@@ -621,7 +621,7 @@
         <v>0.1</v>
       </c>
       <c r="H6" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -629,13 +629,13 @@
         <v>11</v>
       </c>
       <c r="C7" s="5">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="D7" s="5">
-        <v>1.2</v>
+        <v>1.2E-2</v>
       </c>
       <c r="E7" s="5">
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
       <c r="F7" s="5">
         <v>0</v>
@@ -644,7 +644,7 @@
         <v>0.4</v>
       </c>
       <c r="H7" s="5">
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -652,13 +652,13 @@
         <v>12</v>
       </c>
       <c r="C8" s="5">
-        <v>1.1000000000000001</v>
+        <v>0.11000000000000001</v>
       </c>
       <c r="D8" s="5">
-        <v>1.3</v>
+        <v>1.3000000000000001E-2</v>
       </c>
       <c r="E8" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
       <c r="F8" s="5">
         <v>0</v>
@@ -667,7 +667,7 @@
         <v>0.1</v>
       </c>
       <c r="H8" s="5">
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -675,13 +675,13 @@
         <v>13</v>
       </c>
       <c r="C9" s="5">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="D9" s="5">
-        <v>0.4</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="E9" s="5">
-        <v>0.8</v>
+        <v>8.0000000000000016E-2</v>
       </c>
       <c r="F9" s="5">
         <v>0</v>
@@ -690,7 +690,7 @@
         <v>0.2</v>
       </c>
       <c r="H9" s="5">
-        <v>0.1</v>
+        <v>1.0000000000000002E-2</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -698,13 +698,13 @@
         <v>14</v>
       </c>
       <c r="C10" s="5">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
       <c r="D10" s="5">
-        <v>0.5</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="E10" s="5">
-        <v>0.4</v>
+        <v>4.0000000000000008E-2</v>
       </c>
       <c r="F10" s="5">
         <v>0</v>
@@ -713,7 +713,7 @@
         <v>0.7</v>
       </c>
       <c r="H10" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -721,13 +721,13 @@
         <v>15</v>
       </c>
       <c r="C11" s="5">
-        <v>1.2</v>
+        <v>0.12</v>
       </c>
       <c r="D11" s="5">
-        <v>1.5</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="E11" s="5">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="F11" s="5">
         <v>0.2</v>
@@ -736,7 +736,7 @@
         <v>0.2</v>
       </c>
       <c r="H11" s="5">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -744,13 +744,13 @@
         <v>16</v>
       </c>
       <c r="C12" s="5">
-        <v>1.5</v>
+        <v>0.15000000000000002</v>
       </c>
       <c r="D12" s="5">
-        <v>1.8</v>
+        <v>1.8000000000000002E-2</v>
       </c>
       <c r="E12" s="5">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
       <c r="F12" s="5">
         <v>0.2</v>
@@ -759,7 +759,7 @@
         <v>0.2</v>
       </c>
       <c r="H12" s="5">
-        <v>0.8</v>
+        <v>8.0000000000000016E-2</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -767,13 +767,13 @@
         <v>17</v>
       </c>
       <c r="C13" s="5">
-        <v>0.4</v>
+        <v>4.0000000000000008E-2</v>
       </c>
       <c r="D13" s="5">
-        <v>0.3</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="E13" s="5">
-        <v>1.1000000000000001</v>
+        <v>0.11000000000000001</v>
       </c>
       <c r="F13" s="5">
         <v>1.3</v>
@@ -782,7 +782,7 @@
         <v>0.2</v>
       </c>
       <c r="H13" s="5">
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -790,13 +790,13 @@
         <v>18</v>
       </c>
       <c r="C14" s="5">
-        <v>0.8</v>
+        <v>8.0000000000000016E-2</v>
       </c>
       <c r="D14" s="5">
-        <v>0.7</v>
+        <v>6.9999999999999993E-3</v>
       </c>
       <c r="E14" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
       <c r="F14" s="5">
         <v>0</v>
@@ -805,7 +805,7 @@
         <v>0.1</v>
       </c>
       <c r="H14" s="5">
-        <v>0.4</v>
+        <v>4.0000000000000008E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
migrating all scenario files to staging branch
</commit_message>
<xml_diff>
--- a/data/Beacon_Harbor_Winds of Fortune Template.xlsx
+++ b/data/Beacon_Harbor_Winds of Fortune Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Probability Management\Portfolio Build\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F5A095A-CC77-4201-B7A3-EBE7102BBD71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED2FD44-1633-4999-8AF8-926DC0E32420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{62E0E9A3-437D-464E-8FB6-CFA38D87EB32}"/>
   </bookViews>
@@ -583,13 +583,13 @@
         <v>9</v>
       </c>
       <c r="C5" s="5">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
       <c r="D5" s="5">
-        <v>0.5</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="E5" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
       <c r="F5" s="5">
         <v>0</v>
@@ -598,7 +598,7 @@
         <v>0.3</v>
       </c>
       <c r="H5" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -606,13 +606,13 @@
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <v>0.7</v>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="D6" s="5">
-        <v>0.6</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="E6" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
       <c r="F6" s="5">
         <v>0</v>
@@ -621,7 +621,7 @@
         <v>0.1</v>
       </c>
       <c r="H6" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -629,13 +629,13 @@
         <v>11</v>
       </c>
       <c r="C7" s="5">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="D7" s="5">
-        <v>1.2</v>
+        <v>1.2E-2</v>
       </c>
       <c r="E7" s="5">
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
       <c r="F7" s="5">
         <v>0</v>
@@ -644,7 +644,7 @@
         <v>0.4</v>
       </c>
       <c r="H7" s="5">
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -652,13 +652,13 @@
         <v>12</v>
       </c>
       <c r="C8" s="5">
-        <v>1.1000000000000001</v>
+        <v>0.11000000000000001</v>
       </c>
       <c r="D8" s="5">
-        <v>1.3</v>
+        <v>1.3000000000000001E-2</v>
       </c>
       <c r="E8" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
       <c r="F8" s="5">
         <v>0</v>
@@ -667,7 +667,7 @@
         <v>0.1</v>
       </c>
       <c r="H8" s="5">
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -675,13 +675,13 @@
         <v>13</v>
       </c>
       <c r="C9" s="5">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="D9" s="5">
-        <v>0.4</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="E9" s="5">
-        <v>0.8</v>
+        <v>8.0000000000000016E-2</v>
       </c>
       <c r="F9" s="5">
         <v>0</v>
@@ -690,7 +690,7 @@
         <v>0.2</v>
       </c>
       <c r="H9" s="5">
-        <v>0.1</v>
+        <v>1.0000000000000002E-2</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -698,13 +698,13 @@
         <v>14</v>
       </c>
       <c r="C10" s="5">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
       <c r="D10" s="5">
-        <v>0.5</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="E10" s="5">
-        <v>0.4</v>
+        <v>4.0000000000000008E-2</v>
       </c>
       <c r="F10" s="5">
         <v>0</v>
@@ -713,7 +713,7 @@
         <v>0.7</v>
       </c>
       <c r="H10" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -721,13 +721,13 @@
         <v>15</v>
       </c>
       <c r="C11" s="5">
-        <v>1.2</v>
+        <v>0.12</v>
       </c>
       <c r="D11" s="5">
-        <v>1.5</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="E11" s="5">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="F11" s="5">
         <v>0.2</v>
@@ -736,7 +736,7 @@
         <v>0.2</v>
       </c>
       <c r="H11" s="5">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -744,13 +744,13 @@
         <v>16</v>
       </c>
       <c r="C12" s="5">
-        <v>1.5</v>
+        <v>0.15000000000000002</v>
       </c>
       <c r="D12" s="5">
-        <v>1.8</v>
+        <v>1.8000000000000002E-2</v>
       </c>
       <c r="E12" s="5">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
       <c r="F12" s="5">
         <v>0.2</v>
@@ -759,7 +759,7 @@
         <v>0.2</v>
       </c>
       <c r="H12" s="5">
-        <v>0.8</v>
+        <v>8.0000000000000016E-2</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -767,13 +767,13 @@
         <v>17</v>
       </c>
       <c r="C13" s="5">
-        <v>0.4</v>
+        <v>4.0000000000000008E-2</v>
       </c>
       <c r="D13" s="5">
-        <v>0.3</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="E13" s="5">
-        <v>1.1000000000000001</v>
+        <v>0.11000000000000001</v>
       </c>
       <c r="F13" s="5">
         <v>1.3</v>
@@ -782,7 +782,7 @@
         <v>0.2</v>
       </c>
       <c r="H13" s="5">
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -790,13 +790,13 @@
         <v>18</v>
       </c>
       <c r="C14" s="5">
-        <v>0.8</v>
+        <v>8.0000000000000016E-2</v>
       </c>
       <c r="D14" s="5">
-        <v>0.7</v>
+        <v>6.9999999999999993E-3</v>
       </c>
       <c r="E14" s="5">
-        <v>0.2</v>
+        <v>2.0000000000000004E-2</v>
       </c>
       <c r="F14" s="5">
         <v>0</v>
@@ -805,7 +805,7 @@
         <v>0.1</v>
       </c>
       <c r="H14" s="5">
-        <v>0.4</v>
+        <v>4.0000000000000008E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>